<commit_message>
Update RHPF for US scenario assumptions
</commit_message>
<xml_diff>
--- a/InputData/hydgn/RHPF/Recipient Hydrogen Pathway Fractions.xlsx
+++ b/InputData/hydgn/RHPF/Recipient Hydrogen Pathway Fractions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\hydgn\RHPF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8AA43F9-77A7-447F-8C44-DDD7DF7C76CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{067FFBEF-747A-4D2E-AD47-DECE90DD892E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -422,14 +422,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -437,42 +437,42 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>14</v>
       </c>
@@ -489,14 +489,14 @@
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="34.28515625" customWidth="1"/>
-    <col min="2" max="6" width="16.5703125" style="3" customWidth="1"/>
-    <col min="7" max="8" width="16.42578125" customWidth="1"/>
+    <col min="1" max="1" width="34.26953125" customWidth="1"/>
+    <col min="2" max="6" width="16.54296875" style="3" customWidth="1"/>
+    <col min="7" max="8" width="16.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>13</v>
       </c>
@@ -522,7 +522,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -541,40 +541,40 @@
       <c r="F2" s="3">
         <v>0</v>
       </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G2" s="3">
+        <v>0</v>
+      </c>
+      <c r="H2" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C3" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H3" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -600,7 +600,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -626,7 +626,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -652,56 +652,56 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>15</v>
       </c>
       <c r="B7" s="3">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="C7" s="3">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="D7" s="3">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E7" s="3">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="F7" s="3">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="G7" s="3">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="H7" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
       <c r="B8" s="3">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="C8" s="3">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="D8" s="3">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="E8" s="3">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="F8" s="3">
-        <v>0</v>
-      </c>
-      <c r="G8">
-        <v>0</v>
-      </c>
-      <c r="H8">
-        <v>0</v>
+        <v>0.75</v>
+      </c>
+      <c r="G8" s="3">
+        <v>0.75</v>
+      </c>
+      <c r="H8" s="3">
+        <v>0.75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>